<commit_message>
(Set-ExecutionPolicy -Scope Process -ExecutionPolicy RemoteSigned) ; (& c:\Condominio\venv\Scripts\Activate.ps1)
</commit_message>
<xml_diff>
--- a/planilhas/Contabilidade Condominio.xlsx
+++ b/planilhas/Contabilidade Condominio.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Condominio\planilhas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4964A83-0902-4BBA-B6A4-F88C01389AAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64267CF7-3CCC-46BF-B07D-2CDF22BC1374}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CAPA Explicações" sheetId="1" r:id="rId1"/>
@@ -7769,7 +7769,7 @@
       </c>
       <c r="F8" s="61">
         <f t="shared" ref="F8:M8" si="1">SUM(F9:F11)</f>
-        <v>0</v>
+        <v>635.12</v>
       </c>
       <c r="G8" s="61">
         <f t="shared" si="1"/>
@@ -7822,7 +7822,7 @@
       </c>
       <c r="F9" s="63">
         <f>TaxaCondominio!AD10</f>
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="G9" s="63">
         <f>TaxaCondominio!AE10</f>
@@ -7869,7 +7869,9 @@
       <c r="E10" s="65">
         <v>24.97</v>
       </c>
-      <c r="F10" s="66"/>
+      <c r="F10" s="66">
+        <v>35.119999999999997</v>
+      </c>
       <c r="G10" s="66"/>
       <c r="H10" s="65"/>
       <c r="I10" s="65"/>
@@ -8081,7 +8083,7 @@
       </c>
       <c r="F17" s="68">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>976.31</v>
       </c>
       <c r="G17" s="68">
         <f t="shared" si="4"/>
@@ -8129,7 +8131,7 @@
         <v>81.239999999999995</v>
       </c>
       <c r="F18" s="70">
-        <v>0</v>
+        <v>81.239999999999995</v>
       </c>
       <c r="G18" s="70">
         <v>0</v>
@@ -8170,7 +8172,7 @@
         <v>63.67</v>
       </c>
       <c r="F19" s="70">
-        <v>0</v>
+        <v>64.680000000000007</v>
       </c>
       <c r="G19" s="70">
         <v>0</v>
@@ -8211,7 +8213,8 @@
         <v>0</v>
       </c>
       <c r="F20" s="69">
-        <v>0</v>
+        <f>150 + 150 + 399 + 131.39</f>
+        <v>830.39</v>
       </c>
       <c r="G20" s="69">
         <v>0</v>
@@ -8479,7 +8482,8 @@
         <v>3419.26</v>
       </c>
       <c r="F28" s="70">
-        <v>0</v>
+        <f>E33+F8</f>
+        <v>3759.4700000000003</v>
       </c>
       <c r="G28" s="70">
         <v>0</v>
@@ -8577,7 +8581,7 @@
       </c>
       <c r="F30" s="70">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>976.31</v>
       </c>
       <c r="G30" s="70">
         <f t="shared" si="8"/>
@@ -8737,7 +8741,7 @@
       </c>
       <c r="F33" s="73">
         <f t="shared" si="11"/>
-        <v>-150</v>
+        <v>2633.1600000000003</v>
       </c>
       <c r="G33" s="73">
         <f t="shared" si="11"/>
@@ -9910,6 +9914,7 @@
       <c r="AA3" s="82"/>
       <c r="AB3" s="82"/>
       <c r="AC3" s="82"/>
+      <c r="AD3" s="82"/>
     </row>
     <row r="4" spans="1:39" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="78" t="s">
@@ -10011,6 +10016,9 @@
       <c r="AC4" s="84">
         <v>46113</v>
       </c>
+      <c r="AD4" s="84">
+        <v>46143</v>
+      </c>
     </row>
     <row r="5" spans="1:39" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="81">
@@ -10100,6 +10108,9 @@
       <c r="AC5" s="120">
         <v>150</v>
       </c>
+      <c r="AD5" s="120">
+        <v>150</v>
+      </c>
     </row>
     <row r="6" spans="1:39" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="81">
@@ -10189,6 +10200,9 @@
       <c r="AC6" s="89">
         <v>150</v>
       </c>
+      <c r="AD6" s="89">
+        <v>150</v>
+      </c>
     </row>
     <row r="7" spans="1:39" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="81">
@@ -10278,6 +10292,9 @@
       <c r="AC7" s="89">
         <v>150</v>
       </c>
+      <c r="AD7" s="89">
+        <v>150</v>
+      </c>
     </row>
     <row r="8" spans="1:39" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="81">
@@ -10365,6 +10382,9 @@
         <v>150</v>
       </c>
       <c r="AC8" s="89">
+        <v>150</v>
+      </c>
+      <c r="AD8" s="89">
         <v>150</v>
       </c>
     </row>
@@ -10522,7 +10542,11 @@
         <v>600</v>
       </c>
       <c r="AC10" s="91">
-        <f t="shared" ref="AC10" si="2">SUM(AC5:AC8)</f>
+        <f t="shared" ref="AC10:AD10" si="2">SUM(AC5:AC8)</f>
+        <v>600</v>
+      </c>
+      <c r="AD10" s="91">
+        <f t="shared" si="2"/>
         <v>600</v>
       </c>
     </row>

</xml_diff>